<commit_message>
refactor: enhance guardian lifecycle and telegram logic
- Implement graceful termination for background guardian processes during uninstall.
- Apply strict filtering to Telegram notifications, requiring completion of verification tasks.
- Update release metadata and resource builds to v1.0.8-R6.
</commit_message>
<xml_diff>
--- a/public/reports/EVedhika_UBD_Daily_PC_Report.xlsx
+++ b/public/reports/EVedhika_UBD_Daily_PC_Report.xlsx
@@ -433,7 +433,7 @@
         <v>Report Generated At</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-26 17:30:50 IST</v>
+        <v>2026-10-26 19:41:22 IST</v>
       </c>
     </row>
     <row r="5">
@@ -449,7 +449,7 @@
         <v>Total Unique Computers Deployed</v>
       </c>
       <c r="B6">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -457,7 +457,7 @@
         <v>Successful PCs (17/17 Steps Verified)</v>
       </c>
       <c r="B7">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -473,7 +473,7 @@
         <v>Active USB DSC Tokens Verified</v>
       </c>
       <c r="B9">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
@@ -481,7 +481,7 @@
         <v>Deployment Success Rate</v>
       </c>
       <c r="B10" t="str">
-        <v>95%</v>
+        <v>96%</v>
       </c>
     </row>
     <row r="11">
@@ -501,7 +501,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W23"/>
+  <dimension ref="A1:W24"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -604,16 +604,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>EVD-AP-0FF5-9B02</v>
+        <v>EVD-PC-1900-62E8</v>
       </c>
       <c r="C2" t="str">
-        <v>AP-GP-VIZAG-02</v>
+        <v>GP-MANDAL-DESK-1900</v>
       </c>
       <c r="D2" t="str">
-        <v>Bheemunipatnam Mandal Office, Visakhapatnam, AP</v>
+        <v>Mandal Panchayat Office</v>
       </c>
       <c r="E2" t="str">
-        <v>Andhra Pradesh</v>
+        <v>Telangana</v>
       </c>
       <c r="F2" t="str">
         <v>Standard User Mode</v>
@@ -631,43 +631,43 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K2" t="str">
-        <v>Windows 11 Pro</v>
+        <v>Windows 11 Pro (64-Bit)</v>
       </c>
       <c r="L2" t="str">
-        <v>FAILED</v>
+        <v>ISSUE DETECTED (Edge IE Mode &amp; DSC Policy Drift)</v>
       </c>
       <c r="M2">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="N2" t="str">
-        <v>Failed (12/17 Passed)</v>
+        <v>12/17 steps passed (Action Needed)</v>
       </c>
       <c r="O2" t="str">
-        <v>Token Disconnected</v>
+        <v>SmartCard Service Inactive / Edge Policy Drift</v>
       </c>
       <c r="P2" t="str">
         <v>Port 8080 Active</v>
       </c>
       <c r="Q2" t="str">
-        <v>FAIL (Policy Drift)</v>
+        <v>IE5 Quirks Mode Disconnected</v>
       </c>
       <c r="R2" t="str">
-        <v>Zone 2 Active</v>
+        <v>Zone 2 Configured</v>
       </c>
       <c r="S2" t="str">
-        <v>Active</v>
+        <v>Allowed</v>
       </c>
       <c r="T2" t="str">
-        <v>ubd.telangana.gov.in</v>
+        <v>https://ubd.telangana.gov.in</v>
       </c>
       <c r="U2" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="V2" t="str">
-        <v>3:14:34 PM</v>
+        <v>2:08:36 PM</v>
       </c>
       <c r="W2" t="str">
-        <v>E-Vedhika v1.0.8 Audit: Edge IE Mode Policy verification FAILED (IE Quirks Mode disabled in registry policy).</v>
+        <v>UBD Portal Digital Signature Error: Edge IE Mode policy reset by Windows Update &amp; Port 8080 firewall blocked.</v>
       </c>
     </row>
     <row r="3">
@@ -675,16 +675,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>EVD-TS-5503-A106</v>
+        <v>EVD-AP-0FF5-9B02</v>
       </c>
       <c r="C3" t="str">
-        <v>TS-GP-KHAMMAM-01</v>
+        <v>AP-GP-VIZAG-02</v>
       </c>
       <c r="D3" t="str">
-        <v>Khammam Urban Grama Panchayat, Telangana</v>
+        <v>Bheemunipatnam Mandal Office, Visakhapatnam, AP</v>
       </c>
       <c r="E3" t="str">
-        <v>Telangana</v>
+        <v>Andhra Pradesh</v>
       </c>
       <c r="F3" t="str">
         <v>Standard User Mode</v>
@@ -705,22 +705,22 @@
         <v>Windows 11 Pro</v>
       </c>
       <c r="L3" t="str">
-        <v>SUCCESS</v>
+        <v>FAILED</v>
       </c>
       <c r="M3">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="N3" t="str">
-        <v>Passed (17/17)</v>
+        <v>Failed (12/17 Passed)</v>
       </c>
       <c r="O3" t="str">
-        <v>ProxKey SHA256 Connected</v>
+        <v>Token Disconnected</v>
       </c>
       <c r="P3" t="str">
         <v>Port 8080 Active</v>
       </c>
       <c r="Q3" t="str">
-        <v>IE5 Quirks Active</v>
+        <v>FAIL (Policy Drift)</v>
       </c>
       <c r="R3" t="str">
         <v>Zone 2 Active</v>
@@ -738,7 +738,7 @@
         <v>3:14:34 PM</v>
       </c>
       <c r="W3" t="str">
-        <v>17/17 Deployment steps executed and verified with zero manual clicks! 24*7 Guardian Active.</v>
+        <v>E-Vedhika v1.0.8 Audit: Edge IE Mode Policy verification FAILED (IE Quirks Mode disabled in registry policy).</v>
       </c>
     </row>
     <row r="4">
@@ -746,13 +746,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>EVD-TS-7720-7F09</v>
+        <v>EVD-TS-5503-A106</v>
       </c>
       <c r="C4" t="str">
-        <v>GUARDIAN-GP-MANDAL-01</v>
+        <v>TS-GP-KHAMMAM-01</v>
       </c>
       <c r="D4" t="str">
-        <v>Khammam Mandal Office (Telangana)</v>
+        <v>Khammam Urban Grama Panchayat, Telangana</v>
       </c>
       <c r="E4" t="str">
         <v>Telangana</v>
@@ -761,19 +761,19 @@
         <v>Standard User Mode</v>
       </c>
       <c r="G4" t="str">
-        <v>183.82.98.22</v>
+        <v>183.82.98.11</v>
       </c>
       <c r="H4" t="str">
-        <v>16 GB (12.4 GB Free)</v>
+        <v>8.00 GB (4.20 GB Free)</v>
       </c>
       <c r="I4" t="str">
-        <v>180 GB Free</v>
+        <v>120.00 GB Free</v>
       </c>
       <c r="J4" t="str">
-        <v>Intel(R) Core(TM) i7-12700H @ 2.70GHz</v>
+        <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K4" t="str">
-        <v>Windows 11 Pro (Build 22631)</v>
+        <v>Windows 11 Pro</v>
       </c>
       <c r="L4" t="str">
         <v>SUCCESS</v>
@@ -785,28 +785,28 @@
         <v>Passed (17/17)</v>
       </c>
       <c r="O4" t="str">
-        <v>USB Token Connected (ProxKey SHA256)</v>
+        <v>ProxKey SHA256 Connected</v>
       </c>
       <c r="P4" t="str">
         <v>Port 8080 Active</v>
       </c>
       <c r="Q4" t="str">
-        <v>Active</v>
+        <v>IE5 Quirks Active</v>
       </c>
       <c r="R4" t="str">
-        <v>Active</v>
+        <v>Zone 2 Active</v>
       </c>
       <c r="S4" t="str">
         <v>Active</v>
       </c>
       <c r="T4" t="str">
-        <v>https://ubd.telangana.gov.in</v>
+        <v>ubd.telangana.gov.in</v>
       </c>
       <c r="U4" t="str">
         <v>2026-10-25</v>
       </c>
       <c r="V4" t="str">
-        <v>1:39:40 PM</v>
+        <v>3:14:34 PM</v>
       </c>
       <c r="W4" t="str">
         <v>17/17 Deployment steps executed and verified with zero manual clicks! 24*7 Guardian Active.</v>
@@ -817,13 +817,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>EVD-TS-615D-8828</v>
+        <v>EVD-TS-7720-7F09</v>
       </c>
       <c r="C5" t="str">
-        <v>DUMMY-GP-OFFICE-01</v>
+        <v>GUARDIAN-GP-MANDAL-01</v>
       </c>
       <c r="D5" t="str">
-        <v>Suryapet Mandal Office (Telangana)</v>
+        <v>Khammam Mandal Office (Telangana)</v>
       </c>
       <c r="E5" t="str">
         <v>Telangana</v>
@@ -832,16 +832,16 @@
         <v>Standard User Mode</v>
       </c>
       <c r="G5" t="str">
-        <v>183.82.98.11</v>
+        <v>183.82.98.22</v>
       </c>
       <c r="H5" t="str">
-        <v>16 GB (11.2 GB Free)</v>
+        <v>16 GB (12.4 GB Free)</v>
       </c>
       <c r="I5" t="str">
-        <v>240 GB Free</v>
+        <v>180 GB Free</v>
       </c>
       <c r="J5" t="str">
-        <v>12th Gen Intel(R) Core(TM) i7-12700H</v>
+        <v>Intel(R) Core(TM) i7-12700H @ 2.70GHz</v>
       </c>
       <c r="K5" t="str">
         <v>Windows 11 Pro (Build 22631)</v>
@@ -856,7 +856,7 @@
         <v>Passed (17/17)</v>
       </c>
       <c r="O5" t="str">
-        <v>Active</v>
+        <v>USB Token Connected (ProxKey SHA256)</v>
       </c>
       <c r="P5" t="str">
         <v>Port 8080 Active</v>
@@ -871,16 +871,16 @@
         <v>Active</v>
       </c>
       <c r="T5" t="str">
-        <v>ubd.telangana.gov.in</v>
+        <v>https://ubd.telangana.gov.in</v>
       </c>
       <c r="U5" t="str">
         <v>2026-10-25</v>
       </c>
       <c r="V5" t="str">
-        <v>8:55:50 AM</v>
+        <v>1:39:40 PM</v>
       </c>
       <c r="W5" t="str">
-        <v>17/17 Deployment steps executed and verified with zero manual clicks!</v>
+        <v>17/17 Deployment steps executed and verified with zero manual clicks! 24*7 Guardian Active.</v>
       </c>
     </row>
     <row r="6">
@@ -888,16 +888,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>EVD-AP-7D02-6306</v>
+        <v>EVD-TS-615D-8828</v>
       </c>
       <c r="C6" t="str">
-        <v>ROSI</v>
+        <v>DUMMY-GP-OFFICE-01</v>
       </c>
       <c r="D6" t="str">
-        <v>Gajuwaka Mandal Office, AP</v>
+        <v>Suryapet Mandal Office (Telangana)</v>
       </c>
       <c r="E6" t="str">
-        <v>Andhra Pradesh</v>
+        <v>Telangana</v>
       </c>
       <c r="F6" t="str">
         <v>Standard User Mode</v>
@@ -906,52 +906,52 @@
         <v>183.82.98.11</v>
       </c>
       <c r="H6" t="str">
-        <v>8.00 GB (4.20 GB Free)</v>
+        <v>16 GB (11.2 GB Free)</v>
       </c>
       <c r="I6" t="str">
-        <v>120.00 GB Free</v>
+        <v>240 GB Free</v>
       </c>
       <c r="J6" t="str">
-        <v>Intel(R) Core(TM) i5</v>
+        <v>12th Gen Intel(R) Core(TM) i7-12700H</v>
       </c>
       <c r="K6" t="str">
-        <v>Windows 11 Home Single Language (10.0.26300)</v>
+        <v>Windows 11 Pro (Build 22631)</v>
       </c>
       <c r="L6" t="str">
-        <v>RESOLVED (Auto-Healed)</v>
+        <v>SUCCESS</v>
       </c>
       <c r="M6">
         <v>100</v>
       </c>
       <c r="N6" t="str">
-        <v>15/15 Steps Verified</v>
+        <v>Passed (17/17)</v>
       </c>
       <c r="O6" t="str">
-        <v>Connected (Port 8080 Active)</v>
+        <v>Active</v>
       </c>
       <c r="P6" t="str">
         <v>Port 8080 Active</v>
       </c>
       <c r="Q6" t="str">
-        <v>IE5 Quirks Mode Enforced</v>
+        <v>Active</v>
       </c>
       <c r="R6" t="str">
-        <v>Zone 2 Configured (ubd.ap.gov.in)</v>
+        <v>Active</v>
       </c>
       <c r="S6" t="str">
-        <v>Allowed</v>
+        <v>Active</v>
       </c>
       <c r="T6" t="str">
-        <v>ubd.ap.gov.in</v>
+        <v>ubd.telangana.gov.in</v>
       </c>
       <c r="U6" t="str">
-        <v>2026-10-20</v>
+        <v>2026-10-25</v>
       </c>
       <c r="V6" t="str">
-        <v>7:18:58 PM</v>
+        <v>8:55:50 AM</v>
       </c>
       <c r="W6" t="str">
-        <v>🛡️ [AUTOREPAIR GUARDIAN] Auto-healed Edge IE Mode Policy drift. Post-repair check PASSED (Status: RESOLVED).</v>
+        <v>17/17 Deployment steps executed and verified with zero manual clicks!</v>
       </c>
     </row>
     <row r="7">
@@ -959,13 +959,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>EVD-AP-41B1-565E</v>
+        <v>EVD-AP-7D02-6306</v>
       </c>
       <c r="C7" t="str">
-        <v>ROSI-DESK-01</v>
+        <v>ROSI</v>
       </c>
       <c r="D7" t="str">
-        <v>Gajuwaka GP Office, Visakhapatnam</v>
+        <v>Gajuwaka Mandal Office, AP</v>
       </c>
       <c r="E7" t="str">
         <v>Andhra Pradesh</v>
@@ -986,10 +986,10 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K7" t="str">
-        <v>Windows 11 Home Single Language (Build: 10.0.26300)</v>
+        <v>Windows 11 Home Single Language (10.0.26300)</v>
       </c>
       <c r="L7" t="str">
-        <v>ONLINE &amp; READY</v>
+        <v>RESOLVED (Auto-Healed)</v>
       </c>
       <c r="M7">
         <v>100</v>
@@ -998,16 +998,16 @@
         <v>15/15 Steps Verified</v>
       </c>
       <c r="O7" t="str">
-        <v>Connected (ePass2003 / Token Active)</v>
+        <v>Connected (Port 8080 Active)</v>
       </c>
       <c r="P7" t="str">
-        <v>Port 8080 Active &amp; Listening</v>
+        <v>Port 8080 Active</v>
       </c>
       <c r="Q7" t="str">
-        <v>IE5 Quirks Mode Active</v>
+        <v>IE5 Quirks Mode Enforced</v>
       </c>
       <c r="R7" t="str">
-        <v>Zone 2 Configured (ubd.ap.gov.in &amp; ubd.telangana.gov.in)</v>
+        <v>Zone 2 Configured (ubd.ap.gov.in)</v>
       </c>
       <c r="S7" t="str">
         <v>Allowed</v>
@@ -1019,10 +1019,10 @@
         <v>2026-10-20</v>
       </c>
       <c r="V7" t="str">
-        <v>7:18:52 PM</v>
+        <v>7:18:58 PM</v>
       </c>
       <c r="W7" t="str">
-        <v>✅ [CENTRAL CLOUD LIVE TEST] E-Vedhika v1.0.7: All 15/15 Steps Verified. System 100% Online, Token Active &amp; IE5 Quirks Configured.</v>
+        <v>🛡️ [AUTOREPAIR GUARDIAN] Auto-healed Edge IE Mode Policy drift. Post-repair check PASSED (Status: RESOLVED).</v>
       </c>
     </row>
     <row r="8">
@@ -1030,13 +1030,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>EVD-AP-27A0-C5D6</v>
+        <v>EVD-AP-41B1-565E</v>
       </c>
       <c r="C8" t="str">
-        <v>ROSI</v>
+        <v>ROSI-DESK-01</v>
       </c>
       <c r="D8" t="str">
-        <v>Gajuwaka, Andhra Pradesh</v>
+        <v>Gajuwaka GP Office, Visakhapatnam</v>
       </c>
       <c r="E8" t="str">
         <v>Andhra Pradesh</v>
@@ -1069,16 +1069,16 @@
         <v>15/15 Steps Verified</v>
       </c>
       <c r="O8" t="str">
-        <v>Connected &amp; Active (Port 8080)</v>
+        <v>Connected (ePass2003 / Token Active)</v>
       </c>
       <c r="P8" t="str">
-        <v>Port 8080 Active</v>
+        <v>Port 8080 Active &amp; Listening</v>
       </c>
       <c r="Q8" t="str">
         <v>IE5 Quirks Mode Active</v>
       </c>
       <c r="R8" t="str">
-        <v>Zone 2 Configured (ubd.ap.gov.in)</v>
+        <v>Zone 2 Configured (ubd.ap.gov.in &amp; ubd.telangana.gov.in)</v>
       </c>
       <c r="S8" t="str">
         <v>Allowed</v>
@@ -1090,10 +1090,10 @@
         <v>2026-10-20</v>
       </c>
       <c r="V8" t="str">
-        <v>7:01:23 PM</v>
+        <v>7:18:52 PM</v>
       </c>
       <c r="W8" t="str">
-        <v>✅ Dummy Test Report: E-Vedhika v1.0.7 All 15/15 Steps Verified. System 100% Online &amp; Ready.</v>
+        <v>✅ [CENTRAL CLOUD LIVE TEST] E-Vedhika v1.0.7: All 15/15 Steps Verified. System 100% Online, Token Active &amp; IE5 Quirks Configured.</v>
       </c>
     </row>
     <row r="9">
@@ -1101,16 +1101,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>EVD-TS-79B7-CABD</v>
+        <v>EVD-AP-27A0-C5D6</v>
       </c>
       <c r="C9" t="str">
-        <v>TEST-GP-PC</v>
+        <v>ROSI</v>
       </c>
       <c r="D9" t="str">
-        <v>Rangareddy, Telangana</v>
+        <v>Gajuwaka, Andhra Pradesh</v>
       </c>
       <c r="E9" t="str">
-        <v>Telangana</v>
+        <v>Andhra Pradesh</v>
       </c>
       <c r="F9" t="str">
         <v>Standard User Mode</v>
@@ -1128,43 +1128,43 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K9" t="str">
-        <v>Win11 Pro (64-Bit)</v>
+        <v>Windows 11 Home Single Language (Build: 10.0.26300)</v>
       </c>
       <c r="L9" t="str">
-        <v>SUCCESS</v>
+        <v>ONLINE &amp; READY</v>
       </c>
       <c r="M9">
         <v>100</v>
       </c>
       <c r="N9" t="str">
-        <v>Passed (15/15)</v>
+        <v>15/15 Steps Verified</v>
       </c>
       <c r="O9" t="str">
-        <v>USB Token Driver Active</v>
+        <v>Connected &amp; Active (Port 8080)</v>
       </c>
       <c r="P9" t="str">
         <v>Port 8080 Active</v>
       </c>
       <c r="Q9" t="str">
-        <v>IE5 Quirks Active</v>
+        <v>IE5 Quirks Mode Active</v>
       </c>
       <c r="R9" t="str">
-        <v>Zone 2 Configured (ubd.telangana.gov.in)</v>
+        <v>Zone 2 Configured (ubd.ap.gov.in)</v>
       </c>
       <c r="S9" t="str">
         <v>Allowed</v>
       </c>
       <c r="T9" t="str">
-        <v>ubd.telangana.gov.in</v>
+        <v>ubd.ap.gov.in</v>
       </c>
       <c r="U9" t="str">
-        <v>2026-10-17</v>
+        <v>2026-10-20</v>
       </c>
       <c r="V9" t="str">
-        <v>3:28:38 PM</v>
+        <v>7:01:23 PM</v>
       </c>
       <c r="W9" t="str">
-        <v>Report received successfully.</v>
+        <v>✅ Dummy Test Report: E-Vedhika v1.0.7 All 15/15 Steps Verified. System 100% Online &amp; Ready.</v>
       </c>
     </row>
     <row r="10">
@@ -1172,13 +1172,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>EVD-PC-XXXX</v>
+        <v>EVD-TS-79B7-CABD</v>
       </c>
       <c r="C10" t="str">
-        <v>GP-WARANGAL-01</v>
+        <v>TEST-GP-PC</v>
       </c>
       <c r="D10" t="str">
-        <v>Hanamkonda Grama Panchayat</v>
+        <v>Rangareddy, Telangana</v>
       </c>
       <c r="E10" t="str">
         <v>Telangana</v>
@@ -1199,16 +1199,16 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K10" t="str">
-        <v>Windows 10/11</v>
+        <v>Win11 Pro (64-Bit)</v>
       </c>
       <c r="L10" t="str">
-        <v>UBD ISSUE AUTO-REPORTED</v>
+        <v>SUCCESS</v>
       </c>
       <c r="M10">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="N10" t="str">
-        <v>Auto Bug Logged</v>
+        <v>Passed (15/15)</v>
       </c>
       <c r="O10" t="str">
         <v>USB Token Driver Active</v>
@@ -1220,22 +1220,22 @@
         <v>IE5 Quirks Active</v>
       </c>
       <c r="R10" t="str">
-        <v>Zone 2 Configured</v>
+        <v>Zone 2 Configured (ubd.telangana.gov.in)</v>
       </c>
       <c r="S10" t="str">
         <v>Allowed</v>
       </c>
       <c r="T10" t="str">
-        <v>https://ubd.telangana.gov.in</v>
+        <v>ubd.telangana.gov.in</v>
       </c>
       <c r="U10" t="str">
         <v>2026-10-17</v>
       </c>
       <c r="V10" t="str">
-        <v>11:44:12 AM</v>
+        <v>3:28:38 PM</v>
       </c>
       <c r="W10" t="str">
-        <v>[UBD-ISSUE] Test UBD Verification Issue: ActiveX initialized successfully for Zone 2. Test diagnostic report.</v>
+        <v>Report received successfully.</v>
       </c>
     </row>
     <row r="11">
@@ -1243,16 +1243,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>EVD-AP-4E67-2E69</v>
+        <v>EVD-PC-XXXX</v>
       </c>
       <c r="C11" t="str">
-        <v>AP-GP-VIZAG-02</v>
+        <v>GP-WARANGAL-01</v>
       </c>
       <c r="D11" t="str">
-        <v>Bheemunipatnam Mandal Office, Visakhapatnam, AP</v>
+        <v>Hanamkonda Grama Panchayat</v>
       </c>
       <c r="E11" t="str">
-        <v>Andhra Pradesh</v>
+        <v>Telangana</v>
       </c>
       <c r="F11" t="str">
         <v>Standard User Mode</v>
@@ -1270,19 +1270,19 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K11" t="str">
-        <v>Win11 Pro (64-Bit)</v>
+        <v>Windows 10/11</v>
       </c>
       <c r="L11" t="str">
-        <v>SUCCESS</v>
+        <v>UBD ISSUE AUTO-REPORTED</v>
       </c>
       <c r="M11">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="N11" t="str">
-        <v>16/16 Passed (48/48 Registry Keys)</v>
+        <v>Auto Bug Logged</v>
       </c>
       <c r="O11" t="str">
-        <v>HYP2003 ePass Token Connected</v>
+        <v>USB Token Driver Active</v>
       </c>
       <c r="P11" t="str">
         <v>Port 8080 Active</v>
@@ -1291,22 +1291,22 @@
         <v>IE5 Quirks Active</v>
       </c>
       <c r="R11" t="str">
-        <v>Zone 2 Configured (ubd.ap.gov.in)</v>
+        <v>Zone 2 Configured</v>
       </c>
       <c r="S11" t="str">
         <v>Allowed</v>
       </c>
       <c r="T11" t="str">
-        <v>ubd.ap.gov.in</v>
+        <v>https://ubd.telangana.gov.in</v>
       </c>
       <c r="U11" t="str">
-        <v>2026-10-16</v>
+        <v>2026-10-17</v>
       </c>
       <c r="V11" t="str">
-        <v>7:15:46 PM</v>
+        <v>11:44:12 AM</v>
       </c>
       <c r="W11" t="str">
-        <v>Deployment Successful - Ready for UBD Portal [GATEWAY: /api/telemetry]</v>
+        <v>[UBD-ISSUE] Test UBD Verification Issue: ActiveX initialized successfully for Zone 2. Test diagnostic report.</v>
       </c>
     </row>
     <row r="12">
@@ -1314,16 +1314,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>EVD-TS-5BA8-4B80</v>
+        <v>EVD-AP-4E67-2E69</v>
       </c>
       <c r="C12" t="str">
-        <v>TS-GP-KHAMMAM-01</v>
+        <v>AP-GP-VIZAG-02</v>
       </c>
       <c r="D12" t="str">
-        <v>Khammam Urban Grama Panchayat, Telangana</v>
+        <v>Bheemunipatnam Mandal Office, Visakhapatnam, AP</v>
       </c>
       <c r="E12" t="str">
-        <v>Telangana</v>
+        <v>Andhra Pradesh</v>
       </c>
       <c r="F12" t="str">
         <v>Standard User Mode</v>
@@ -1341,7 +1341,7 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K12" t="str">
-        <v>Windows 10/11</v>
+        <v>Win11 Pro (64-Bit)</v>
       </c>
       <c r="L12" t="str">
         <v>SUCCESS</v>
@@ -1353,7 +1353,7 @@
         <v>16/16 Passed (48/48 Registry Keys)</v>
       </c>
       <c r="O12" t="str">
-        <v>ProxKey USB Token Connected</v>
+        <v>HYP2003 ePass Token Connected</v>
       </c>
       <c r="P12" t="str">
         <v>Port 8080 Active</v>
@@ -1362,22 +1362,22 @@
         <v>IE5 Quirks Active</v>
       </c>
       <c r="R12" t="str">
-        <v>Zone 2 Configured</v>
+        <v>Zone 2 Configured (ubd.ap.gov.in)</v>
       </c>
       <c r="S12" t="str">
         <v>Allowed</v>
       </c>
       <c r="T12" t="str">
-        <v>ubd.telangana.gov.in</v>
+        <v>ubd.ap.gov.in</v>
       </c>
       <c r="U12" t="str">
         <v>2026-10-16</v>
       </c>
       <c r="V12" t="str">
-        <v>7:15:45 PM</v>
+        <v>7:15:46 PM</v>
       </c>
       <c r="W12" t="str">
-        <v>Deployment Successful - Ready for UBD Portal [GATEWAY: /admin/exe_ubd_live]</v>
+        <v>Deployment Successful - Ready for UBD Portal [GATEWAY: /api/telemetry]</v>
       </c>
     </row>
     <row r="13">
@@ -1385,13 +1385,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>EVD-TS-4A9B-12EF</v>
+        <v>EVD-TS-5BA8-4B80</v>
       </c>
       <c r="C13" t="str">
         <v>TS-GP-KHAMMAM-01</v>
       </c>
       <c r="D13" t="str">
-        <v>Khammam Urban Grama Panchayat</v>
+        <v>Khammam Urban Grama Panchayat, Telangana</v>
       </c>
       <c r="E13" t="str">
         <v>Telangana</v>
@@ -1412,7 +1412,7 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K13" t="str">
-        <v>Windows 11 Pro (64-Bit)</v>
+        <v>Windows 10/11</v>
       </c>
       <c r="L13" t="str">
         <v>SUCCESS</v>
@@ -1421,19 +1421,19 @@
         <v>100</v>
       </c>
       <c r="N13" t="str">
-        <v>16/16 Passed (48/48 Registry Keys Configured)</v>
+        <v>16/16 Passed (48/48 Registry Keys)</v>
       </c>
       <c r="O13" t="str">
         <v>ProxKey USB Token Connected</v>
       </c>
       <c r="P13" t="str">
-        <v>Port 8080 Active (DigiSignHelper Registered)</v>
+        <v>Port 8080 Active</v>
       </c>
       <c r="Q13" t="str">
-        <v>IE5 Quirks Mode Active</v>
+        <v>IE5 Quirks Active</v>
       </c>
       <c r="R13" t="str">
-        <v>Zone 2 Configured (ubd.telangana.gov.in)</v>
+        <v>Zone 2 Configured</v>
       </c>
       <c r="S13" t="str">
         <v>Allowed</v>
@@ -1445,7 +1445,7 @@
         <v>2026-10-16</v>
       </c>
       <c r="V13" t="str">
-        <v>12:45:10 PM</v>
+        <v>7:15:45 PM</v>
       </c>
       <c r="W13" t="str">
         <v>Deployment Successful - Ready for UBD Portal [GATEWAY: /admin/exe_ubd_live]</v>
@@ -1456,16 +1456,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>EVD-AP-88F3-90CC</v>
+        <v>EVD-TS-4A9B-12EF</v>
       </c>
       <c r="C14" t="str">
-        <v>AP-GP-VIZAG-02</v>
+        <v>TS-GP-KHAMMAM-01</v>
       </c>
       <c r="D14" t="str">
-        <v>Bheemunipatnam Mandal Office, Visakhapatnam</v>
+        <v>Khammam Urban Grama Panchayat</v>
       </c>
       <c r="E14" t="str">
-        <v>Andhra Pradesh</v>
+        <v>Telangana</v>
       </c>
       <c r="F14" t="str">
         <v>Standard User Mode</v>
@@ -1483,7 +1483,7 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K14" t="str">
-        <v>Windows 10 Pro (64-Bit)</v>
+        <v>Windows 11 Pro (64-Bit)</v>
       </c>
       <c r="L14" t="str">
         <v>SUCCESS</v>
@@ -1495,31 +1495,31 @@
         <v>16/16 Passed (48/48 Registry Keys Configured)</v>
       </c>
       <c r="O14" t="str">
-        <v>HYP2003 ePass Token Connected</v>
+        <v>ProxKey USB Token Connected</v>
       </c>
       <c r="P14" t="str">
-        <v>Port 8080 Active</v>
+        <v>Port 8080 Active (DigiSignHelper Registered)</v>
       </c>
       <c r="Q14" t="str">
         <v>IE5 Quirks Mode Active</v>
       </c>
       <c r="R14" t="str">
-        <v>Zone 2 Configured (ubd.ap.gov.in)</v>
+        <v>Zone 2 Configured (ubd.telangana.gov.in)</v>
       </c>
       <c r="S14" t="str">
         <v>Allowed</v>
       </c>
       <c r="T14" t="str">
-        <v>ubd.ap.gov.in</v>
+        <v>ubd.telangana.gov.in</v>
       </c>
       <c r="U14" t="str">
         <v>2026-10-16</v>
       </c>
       <c r="V14" t="str">
-        <v>12:44:25 PM</v>
+        <v>12:45:10 PM</v>
       </c>
       <c r="W14" t="str">
-        <v>Deployment Successful - Ready for UBD Portal [GATEWAY: /api/telemetry]</v>
+        <v>Deployment Successful - Ready for UBD Portal [GATEWAY: /admin/exe_ubd_live]</v>
       </c>
     </row>
     <row r="15">
@@ -1527,16 +1527,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>EVD-PC-XXXX</v>
+        <v>EVD-AP-88F3-90CC</v>
       </c>
       <c r="C15" t="str">
-        <v>GP-PC-AUTO-01</v>
+        <v>AP-GP-VIZAG-02</v>
       </c>
       <c r="D15" t="str">
-        <v>Siddipet, Telangana</v>
+        <v>Bheemunipatnam Mandal Office, Visakhapatnam</v>
       </c>
       <c r="E15" t="str">
-        <v>Telangana</v>
+        <v>Andhra Pradesh</v>
       </c>
       <c r="F15" t="str">
         <v>Standard User Mode</v>
@@ -1554,43 +1554,43 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K15" t="str">
-        <v>Windows 10/11</v>
+        <v>Windows 10 Pro (64-Bit)</v>
       </c>
       <c r="L15" t="str">
-        <v>UBD ISSUE AUTO-REPORTED</v>
+        <v>SUCCESS</v>
       </c>
       <c r="M15">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="N15" t="str">
-        <v>Auto Bug Logged</v>
+        <v>16/16 Passed (48/48 Registry Keys Configured)</v>
       </c>
       <c r="O15" t="str">
-        <v>ePass2003 Connected</v>
+        <v>HYP2003 ePass Token Connected</v>
       </c>
       <c r="P15" t="str">
         <v>Port 8080 Active</v>
       </c>
       <c r="Q15" t="str">
-        <v>IE5 Quirks Active</v>
+        <v>IE5 Quirks Mode Active</v>
       </c>
       <c r="R15" t="str">
-        <v>Zone 2 Configured</v>
+        <v>Zone 2 Configured (ubd.ap.gov.in)</v>
       </c>
       <c r="S15" t="str">
         <v>Allowed</v>
       </c>
       <c r="T15" t="str">
-        <v>https://ubd.telangana.gov.in</v>
+        <v>ubd.ap.gov.in</v>
       </c>
       <c r="U15" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-16</v>
       </c>
       <c r="V15" t="str">
-        <v>10:13:35 AM</v>
+        <v>12:44:25 PM</v>
       </c>
       <c r="W15" t="str">
-        <v>[UBD-ISSUE] Silent Background Token Test: Autonomous telemetry test with zero user permissions</v>
+        <v>Deployment Successful - Ready for UBD Portal [GATEWAY: /api/telemetry]</v>
       </c>
     </row>
     <row r="16">
@@ -1601,10 +1601,10 @@
         <v>EVD-PC-XXXX</v>
       </c>
       <c r="C16" t="str">
-        <v>GP-PC-TEST-01</v>
+        <v>GP-PC-AUTO-01</v>
       </c>
       <c r="D16" t="str">
-        <v>Warangal, Telangana</v>
+        <v>Siddipet, Telangana</v>
       </c>
       <c r="E16" t="str">
         <v>Telangana</v>
@@ -1628,16 +1628,16 @@
         <v>Windows 10/11</v>
       </c>
       <c r="L16" t="str">
-        <v>UBD ISSUE REPORTED</v>
+        <v>UBD ISSUE AUTO-REPORTED</v>
       </c>
       <c r="M16">
         <v>65</v>
       </c>
       <c r="N16" t="str">
-        <v>Bug Logged</v>
+        <v>Auto Bug Logged</v>
       </c>
       <c r="O16" t="str">
-        <v>Connected</v>
+        <v>ePass2003 Connected</v>
       </c>
       <c r="P16" t="str">
         <v>Port 8080 Active</v>
@@ -1658,10 +1658,10 @@
         <v>2026-10-09</v>
       </c>
       <c r="V16" t="str">
-        <v>10:05:58 AM</v>
+        <v>10:13:35 AM</v>
       </c>
       <c r="W16" t="str">
-        <v>[UBD-ISSUE] Test DSC Token Verification Error: Test issue description</v>
+        <v>[UBD-ISSUE] Silent Background Token Test: Autonomous telemetry test with zero user permissions</v>
       </c>
     </row>
     <row r="17">
@@ -1669,13 +1669,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>EVD-TS-79A1-606B</v>
+        <v>EVD-PC-XXXX</v>
       </c>
       <c r="C17" t="str">
-        <v>DEBUG-PC-99</v>
+        <v>GP-PC-TEST-01</v>
       </c>
       <c r="D17" t="str">
-        <v>Rangareddy, Telangana</v>
+        <v>Warangal, Telangana</v>
       </c>
       <c r="E17" t="str">
         <v>Telangana</v>
@@ -1696,19 +1696,19 @@
         <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K17" t="str">
-        <v>Win11 Pro (64-Bit)</v>
+        <v>Windows 10/11</v>
       </c>
       <c r="L17" t="str">
-        <v>SUCCESS</v>
+        <v>UBD ISSUE REPORTED</v>
       </c>
       <c r="M17">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="N17" t="str">
-        <v>Passed (15/15)</v>
+        <v>Bug Logged</v>
       </c>
       <c r="O17" t="str">
-        <v>USB Token Driver Active</v>
+        <v>Connected</v>
       </c>
       <c r="P17" t="str">
         <v>Port 8080 Active</v>
@@ -1717,22 +1717,22 @@
         <v>IE5 Quirks Active</v>
       </c>
       <c r="R17" t="str">
-        <v>Zone 2 Configured (ubd.telangana.gov.in)</v>
+        <v>Zone 2 Configured</v>
       </c>
       <c r="S17" t="str">
         <v>Allowed</v>
       </c>
       <c r="T17" t="str">
-        <v>ubd.telangana.gov.in</v>
+        <v>https://ubd.telangana.gov.in</v>
       </c>
       <c r="U17" t="str">
-        <v>2026-10-05</v>
+        <v>2026-10-09</v>
       </c>
       <c r="V17" t="str">
-        <v>4:38:37 PM</v>
+        <v>10:05:58 AM</v>
       </c>
       <c r="W17" t="str">
-        <v>Debugging the admin panel reporting issue.</v>
+        <v>[UBD-ISSUE] Test DSC Token Verification Error: Test issue description</v>
       </c>
     </row>
     <row r="18">
@@ -1740,13 +1740,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>EVD-PC-XXXX</v>
+        <v>EVD-TS-79A1-606B</v>
       </c>
       <c r="C18" t="str">
-        <v>WARANGAL-GP-01</v>
+        <v>DEBUG-PC-99</v>
       </c>
       <c r="D18" t="str">
-        <v>Warangal Mandal Office</v>
+        <v>Rangareddy, Telangana</v>
       </c>
       <c r="E18" t="str">
         <v>Telangana</v>
@@ -1788,22 +1788,22 @@
         <v>IE5 Quirks Active</v>
       </c>
       <c r="R18" t="str">
-        <v>Zone 2 Configured</v>
+        <v>Zone 2 Configured (ubd.telangana.gov.in)</v>
       </c>
       <c r="S18" t="str">
         <v>Allowed</v>
       </c>
       <c r="T18" t="str">
-        <v>https://ubd.telangana.gov.in</v>
+        <v>ubd.telangana.gov.in</v>
       </c>
       <c r="U18" t="str">
-        <v>2026-09-12</v>
+        <v>2026-10-05</v>
       </c>
       <c r="V18" t="str">
-        <v>10:59:24 AM</v>
+        <v>4:38:37 PM</v>
       </c>
       <c r="W18" t="str">
-        <v>Auto-verified Edge IE5 Quirks and DSC Token</v>
+        <v>Debugging the admin panel reporting issue.</v>
       </c>
     </row>
     <row r="19">
@@ -1814,10 +1814,10 @@
         <v>EVD-PC-XXXX</v>
       </c>
       <c r="C19" t="str">
-        <v>TS-PANCHAYAT-SEC-01</v>
+        <v>WARANGAL-GP-01</v>
       </c>
       <c r="D19" t="str">
-        <v>Hanamkonda Grama Panchayat</v>
+        <v>Warangal Mandal Office</v>
       </c>
       <c r="E19" t="str">
         <v>Telangana</v>
@@ -1871,10 +1871,10 @@
         <v>2026-09-12</v>
       </c>
       <c r="V19" t="str">
-        <v>10:59:11 AM</v>
+        <v>10:59:24 AM</v>
       </c>
       <c r="W19" t="str">
-        <v>Edge IE5 Quirks and DSC Token successfully configured</v>
+        <v>Auto-verified Edge IE5 Quirks and DSC Token</v>
       </c>
     </row>
     <row r="20">
@@ -1885,10 +1885,10 @@
         <v>EVD-PC-XXXX</v>
       </c>
       <c r="C20" t="str">
-        <v>TEST-PC-TELUGU</v>
+        <v>TS-PANCHAYAT-SEC-01</v>
       </c>
       <c r="D20" t="str">
-        <v>Warangal Grama Panchayat</v>
+        <v>Hanamkonda Grama Panchayat</v>
       </c>
       <c r="E20" t="str">
         <v>Telangana</v>
@@ -1942,10 +1942,10 @@
         <v>2026-09-12</v>
       </c>
       <c r="V20" t="str">
-        <v>10:58:36 AM</v>
+        <v>10:59:11 AM</v>
       </c>
       <c r="W20" t="str">
-        <v>All 90 parameters verified successfully.</v>
+        <v>Edge IE5 Quirks and DSC Token successfully configured</v>
       </c>
     </row>
     <row r="21">
@@ -1956,10 +1956,10 @@
         <v>EVD-PC-XXXX</v>
       </c>
       <c r="C21" t="str">
-        <v>GRAM-PANCHAYAT-WARANGAL-01</v>
+        <v>TEST-PC-TELUGU</v>
       </c>
       <c r="D21" t="str">
-        <v>Warangal Rural Mandal</v>
+        <v>Warangal Grama Panchayat</v>
       </c>
       <c r="E21" t="str">
         <v>Telangana</v>
@@ -2010,10 +2010,10 @@
         <v>https://ubd.telangana.gov.in</v>
       </c>
       <c r="U21" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-12</v>
       </c>
       <c r="V21" t="str">
-        <v>7:20:39 AM</v>
+        <v>10:58:36 AM</v>
       </c>
       <c r="W21" t="str">
         <v>All 90 parameters verified successfully.</v>
@@ -2027,31 +2027,31 @@
         <v>EVD-PC-XXXX</v>
       </c>
       <c r="C22" t="str">
-        <v>TS-SEC-MND-01</v>
+        <v>GRAM-PANCHAYAT-WARANGAL-01</v>
       </c>
       <c r="D22" t="str">
-        <v>Gram Panchayat Office</v>
+        <v>Warangal Rural Mandal</v>
       </c>
       <c r="E22" t="str">
         <v>Telangana</v>
       </c>
       <c r="F22" t="str">
-        <v>Elevated Administrator Mode (UAC Verified)</v>
+        <v>Standard User Mode</v>
       </c>
       <c r="G22" t="str">
-        <v>192.168.1.104</v>
+        <v>183.82.98.11</v>
       </c>
       <c r="H22" t="str">
-        <v>16 GB (11.2 GB Available)</v>
+        <v>8.00 GB (4.20 GB Free)</v>
       </c>
       <c r="I22" t="str">
-        <v>142 GB Free</v>
+        <v>120.00 GB Free</v>
       </c>
       <c r="J22" t="str">
-        <v>Intel Core i5-11500 @ 2.70GHz</v>
+        <v>Intel(R) Core(TM) i5</v>
       </c>
       <c r="K22" t="str">
-        <v>Windows 11 Pro</v>
+        <v>Win11 Pro (64-Bit)</v>
       </c>
       <c r="L22" t="str">
         <v>SUCCESS</v>
@@ -2060,34 +2060,34 @@
         <v>100</v>
       </c>
       <c r="N22" t="str">
-        <v>17/17 steps passed.</v>
+        <v>Passed (15/15)</v>
       </c>
       <c r="O22" t="str">
-        <v>USB Token Connected</v>
+        <v>USB Token Driver Active</v>
       </c>
       <c r="P22" t="str">
         <v>Port 8080 Active</v>
       </c>
       <c r="Q22" t="str">
-        <v>Enabled</v>
+        <v>IE5 Quirks Active</v>
       </c>
       <c r="R22" t="str">
         <v>Zone 2 Configured</v>
       </c>
       <c r="S22" t="str">
-        <v>Unsigned Allowed (Prompt)</v>
+        <v>Allowed</v>
       </c>
       <c r="T22" t="str">
         <v>https://ubd.telangana.gov.in</v>
       </c>
       <c r="U22" t="str">
-        <v>2026-07-31</v>
+        <v>2026-09-04</v>
       </c>
       <c r="V22" t="str">
-        <v>10:42:15</v>
+        <v>7:20:39 AM</v>
       </c>
       <c r="W22" t="str">
-        <v>All 90 parameters verified. Edge IE Mode &amp; USB DSC Token fully operational.</v>
+        <v>All 90 parameters verified successfully.</v>
       </c>
     </row>
     <row r="23">
@@ -2098,7 +2098,7 @@
         <v>EVD-PC-XXXX</v>
       </c>
       <c r="C23" t="str">
-        <v>PANCHAYAT-PC-04</v>
+        <v>TS-SEC-MND-01</v>
       </c>
       <c r="D23" t="str">
         <v>Gram Panchayat Office</v>
@@ -2110,19 +2110,19 @@
         <v>Elevated Administrator Mode (UAC Verified)</v>
       </c>
       <c r="G23" t="str">
-        <v>192.168.2.45</v>
+        <v>192.168.1.104</v>
       </c>
       <c r="H23" t="str">
-        <v>8 GB (4.1 GB Available)</v>
+        <v>16 GB (11.2 GB Available)</v>
       </c>
       <c r="I23" t="str">
-        <v>88 GB Free</v>
+        <v>142 GB Free</v>
       </c>
       <c r="J23" t="str">
-        <v>Intel Core i3-10100 @ 3.60GHz</v>
+        <v>Intel Core i5-11500 @ 2.70GHz</v>
       </c>
       <c r="K23" t="str">
-        <v>Windows 10 Pro</v>
+        <v>Windows 11 Pro</v>
       </c>
       <c r="L23" t="str">
         <v>SUCCESS</v>
@@ -2146,7 +2146,7 @@
         <v>Zone 2 Configured</v>
       </c>
       <c r="S23" t="str">
-        <v>Unsigned Allowed</v>
+        <v>Unsigned Allowed (Prompt)</v>
       </c>
       <c r="T23" t="str">
         <v>https://ubd.telangana.gov.in</v>
@@ -2155,15 +2155,86 @@
         <v>2026-07-31</v>
       </c>
       <c r="V23" t="str">
+        <v>10:42:15</v>
+      </c>
+      <c r="W23" t="str">
+        <v>All 90 parameters verified. Edge IE Mode &amp; USB DSC Token fully operational.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>EVD-PC-XXXX</v>
+      </c>
+      <c r="C24" t="str">
+        <v>PANCHAYAT-PC-04</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Gram Panchayat Office</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Telangana</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Elevated Administrator Mode (UAC Verified)</v>
+      </c>
+      <c r="G24" t="str">
+        <v>192.168.2.45</v>
+      </c>
+      <c r="H24" t="str">
+        <v>8 GB (4.1 GB Available)</v>
+      </c>
+      <c r="I24" t="str">
+        <v>88 GB Free</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Intel Core i3-10100 @ 3.60GHz</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Windows 10 Pro</v>
+      </c>
+      <c r="L24" t="str">
+        <v>SUCCESS</v>
+      </c>
+      <c r="M24">
+        <v>100</v>
+      </c>
+      <c r="N24" t="str">
+        <v>17/17 steps passed.</v>
+      </c>
+      <c r="O24" t="str">
+        <v>USB Token Connected</v>
+      </c>
+      <c r="P24" t="str">
+        <v>Port 8080 Active</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>Enabled</v>
+      </c>
+      <c r="R24" t="str">
+        <v>Zone 2 Configured</v>
+      </c>
+      <c r="S24" t="str">
+        <v>Unsigned Allowed</v>
+      </c>
+      <c r="T24" t="str">
+        <v>https://ubd.telangana.gov.in</v>
+      </c>
+      <c r="U24" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="V24" t="str">
         <v>10:15:02</v>
       </c>
-      <c r="W23" t="str">
+      <c r="W24" t="str">
         <v>Auto-repaired .NET 3.5 framework successfully. Ready for UBD Portal.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>